<commit_message>
Update Sprint 3 backlog
Added my hours to the sprint backlog
</commit_message>
<xml_diff>
--- a/sprints/sprint3/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint3/Sprint Backlog & Burnup Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\Project\Local Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9e6f5ad0d3e00a8/Desktop/Group5SE2/Group5NutritionTracker/sprints/sprint3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF155070-1F4B-4560-8485-B60514D432E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{AF155070-1F4B-4560-8485-B60514D432E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13E973D7-F7F5-470D-9DDD-35B39FED8F81}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="38">
   <si>
     <t>Related User Story</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>Display Daily Stats</t>
+  </si>
+  <si>
+    <t>Update FoodLog Process Client Side</t>
   </si>
 </sst>
 </file>
@@ -414,21 +417,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$34:$K$34</c:f>
+              <c:f>Sheet1!$H$35:$K$35</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -457,21 +460,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$35:$K$35</c:f>
+              <c:f>Sheet1!$H$36:$K$36</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>36.5</c:v>
+                  <c:v>39.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>36.5</c:v>
+                  <c:v>39.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>36.5</c:v>
+                  <c:v>39.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>36.5</c:v>
+                  <c:v>39.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1221,7 +1224,7 @@
     <xdr:to>
       <xdr:col>19</xdr:col>
       <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>176212</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1513,21 +1516,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K42"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" customWidth="1"/>
-    <col min="5" max="5" width="51.42578125" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" customWidth="1"/>
+    <col min="3" max="3" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.54296875" customWidth="1"/>
+    <col min="5" max="5" width="51.453125" customWidth="1"/>
     <col min="6" max="6" width="44" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.81640625" customWidth="1"/>
+    <col min="10" max="10" width="10.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
         <v>9</v>
       </c>
@@ -1556,7 +1559,7 @@
       <c r="J1" s="10"/>
       <c r="K1" s="10"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="12"/>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -1577,12 +1580,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="9"/>
-      <c r="C3" s="6"/>
+      <c r="C3" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="D3" s="9">
         <v>1.1000000000000001</v>
       </c>
@@ -1595,12 +1600,16 @@
       <c r="G3" s="6">
         <v>3</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="H3" s="3">
+        <v>3</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0</v>
+      </c>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>16</v>
       </c>
@@ -1623,12 +1632,14 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B5" s="9"/>
-      <c r="C5" s="6"/>
+      <c r="C5" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="D5" s="9">
         <v>1.2</v>
       </c>
@@ -1636,30 +1647,34 @@
         <v>10</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="G5" s="6">
-        <v>2.5</v>
-      </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="H5" s="3">
+        <v>3</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0</v>
+      </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="6"/>
       <c r="D6" s="9">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G6" s="6">
         <v>2.5</v>
@@ -1669,9 +1684,9 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="6"/>
@@ -1682,42 +1697,48 @@
         <v>10</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="G7" s="6">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" s="9"/>
-      <c r="C8" s="6"/>
+      <c r="C8" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="D8" s="9">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G8" s="6">
         <v>3</v>
       </c>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
+      <c r="H8" s="3">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
+        <v>2</v>
+      </c>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="6"/>
@@ -1728,68 +1749,70 @@
         <v>36</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G9" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="6"/>
       <c r="D10" s="9">
-        <v>2.2000000000000002</v>
+        <v>2.1</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>36</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G10" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="6"/>
       <c r="D11" s="9">
-        <v>3.1</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G11" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B12" s="9"/>
-      <c r="C12" s="6"/>
+      <c r="C12" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="D12" s="9">
         <v>3.1</v>
       </c>
@@ -1797,19 +1820,23 @@
         <v>24</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G12" s="6">
-        <v>2.5</v>
-      </c>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+        <v>5</v>
+      </c>
+      <c r="H12" s="3">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3">
+        <v>3</v>
+      </c>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="6"/>
@@ -1820,7 +1847,7 @@
         <v>24</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G13" s="6">
         <v>2.5</v>
@@ -1830,9 +1857,9 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="6"/>
@@ -1843,53 +1870,75 @@
         <v>24</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G14" s="6">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B15" s="9"/>
-      <c r="C15" s="6"/>
+      <c r="C15" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="D15" s="9">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>24</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G15" s="6">
-        <v>3</v>
-      </c>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="H15" s="3">
+        <v>0</v>
+      </c>
+      <c r="I15" s="3">
+        <v>2</v>
+      </c>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="6"/>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
+        <v>17</v>
+      </c>
       <c r="B16" s="9"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
+      <c r="C16" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="9">
+        <v>3.2</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="6">
+        <v>3</v>
+      </c>
+      <c r="H16" s="3">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3">
+        <v>2</v>
+      </c>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="6"/>
       <c r="B17" s="9"/>
       <c r="C17" s="6"/>
@@ -1902,7 +1951,7 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="6"/>
       <c r="B18" s="9"/>
       <c r="C18" s="6"/>
@@ -1915,7 +1964,7 @@
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="6"/>
       <c r="B19" s="9"/>
       <c r="C19" s="6"/>
@@ -1928,7 +1977,7 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="6"/>
       <c r="B20" s="9"/>
       <c r="C20" s="6"/>
@@ -1941,7 +1990,7 @@
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="6"/>
       <c r="B21" s="9"/>
       <c r="C21" s="6"/>
@@ -1954,7 +2003,7 @@
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="6"/>
       <c r="B22" s="9"/>
       <c r="C22" s="6"/>
@@ -1967,7 +2016,7 @@
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="6"/>
       <c r="B23" s="9"/>
       <c r="C23" s="6"/>
@@ -1980,7 +2029,7 @@
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="6"/>
       <c r="B24" s="9"/>
       <c r="C24" s="6"/>
@@ -1993,7 +2042,7 @@
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="6"/>
       <c r="B25" s="9"/>
       <c r="C25" s="6"/>
@@ -2006,7 +2055,7 @@
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
       <c r="B26" s="9"/>
       <c r="C26" s="6"/>
@@ -2019,7 +2068,7 @@
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="6"/>
       <c r="B27" s="9"/>
       <c r="C27" s="6"/>
@@ -2032,7 +2081,7 @@
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="6"/>
       <c r="B28" s="9"/>
       <c r="C28" s="6"/>
@@ -2045,7 +2094,7 @@
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="6"/>
       <c r="B29" s="9"/>
       <c r="C29" s="6"/>
@@ -2058,7 +2107,7 @@
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="6"/>
       <c r="B30" s="9"/>
       <c r="C30" s="6"/>
@@ -2071,7 +2120,7 @@
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="6"/>
       <c r="B31" s="9"/>
       <c r="C31" s="6"/>
@@ -2084,7 +2133,7 @@
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="6"/>
       <c r="B32" s="9"/>
       <c r="C32" s="6"/>
@@ -2097,7 +2146,7 @@
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="6"/>
       <c r="B33" s="9"/>
       <c r="C33" s="6"/>
@@ -2110,140 +2159,153 @@
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="4" t="s">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34" s="6"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G34" s="5">
-        <f>SUM(G3:G33)</f>
-        <v>36.5</v>
-      </c>
-      <c r="H34" s="5">
-        <f>SUM(H3:H33)</f>
-        <v>0</v>
-      </c>
-      <c r="I34" s="5">
-        <f>SUM(I3:I33, H34)</f>
-        <v>0</v>
-      </c>
-      <c r="J34" s="5">
-        <f>SUM(J3:J33, I34)</f>
-        <v>0</v>
-      </c>
-      <c r="K34" s="5">
-        <f>SUM(K3:K33, J34)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="G35">
+      <c r="G35" s="5">
+        <f>SUM(G3:G34)</f>
+        <v>39.5</v>
+      </c>
+      <c r="H35" s="5">
+        <f>SUM(H3:H34)</f>
+        <v>6</v>
+      </c>
+      <c r="I35" s="5">
+        <f>SUM(I3:I34, H35)</f>
+        <v>15</v>
+      </c>
+      <c r="J35" s="5">
+        <f>SUM(J3:J34, I35)</f>
+        <v>15</v>
+      </c>
+      <c r="K35" s="5">
+        <f>SUM(K3:K34, J35)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G36">
         <v>96</v>
       </c>
-      <c r="H35">
-        <f>$G$34</f>
-        <v>36.5</v>
-      </c>
-      <c r="I35">
-        <f t="shared" ref="I35:K35" si="0">$G$34</f>
-        <v>36.5</v>
-      </c>
-      <c r="J35">
+      <c r="H36">
+        <f>$G$35</f>
+        <v>39.5</v>
+      </c>
+      <c r="I36">
+        <f t="shared" ref="I36:K36" si="0">$G$35</f>
+        <v>39.5</v>
+      </c>
+      <c r="J36">
         <f t="shared" si="0"/>
-        <v>36.5</v>
-      </c>
-      <c r="K35">
+        <v>39.5</v>
+      </c>
+      <c r="K36">
         <f t="shared" si="0"/>
-        <v>36.5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="F37" s="7" t="s">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="F38" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="G37" s="7" t="s">
+      <c r="G38" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H37" s="8" t="s">
+      <c r="H38" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I37" s="7" t="s">
+      <c r="I38" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="J37" s="8"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F38" t="s">
+      <c r="J38" s="8"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F39" t="s">
         <v>16</v>
       </c>
-      <c r="G38">
-        <f>SUMIF(A3:A33, F38,G3:G33)</f>
+      <c r="G39">
+        <f>SUMIF(A3:A34, F39,G3:G34)</f>
         <v>8</v>
-      </c>
-      <c r="H38">
-        <v>10</v>
-      </c>
-      <c r="I38">
-        <f>H38-G38-G42</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F39" t="s">
-        <v>17</v>
-      </c>
-      <c r="G39">
-        <f>SUMIF(A3:A33, F39,G3:G33)</f>
-        <v>10</v>
       </c>
       <c r="H39">
         <v>10</v>
       </c>
       <c r="I39">
-        <f>H39-G39-G42</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+        <f>H39-G39-G43</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F40" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G40">
-        <f>SUMIF(A3:A33, F40,G3:G33)</f>
-        <v>9</v>
+        <f>SUMIF(A3:A34, F40,G3:G34)</f>
+        <v>10</v>
       </c>
       <c r="H40">
         <v>10</v>
       </c>
       <c r="I40">
-        <f>H40-G40-G42</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+        <f>H40-G40-G43</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F41" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G41">
-        <f>SUMIF(A3:A33, F41,G3:G33)</f>
-        <v>9.5</v>
+        <f>SUMIF(A3:A34, F41,G3:G34)</f>
+        <v>12</v>
       </c>
       <c r="H41">
         <v>10</v>
       </c>
       <c r="I41">
-        <f>H41-G41-G42</f>
+        <f>H41-G41-G43</f>
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="F42" t="s">
+        <v>18</v>
+      </c>
+      <c r="G42">
+        <f>SUMIF(A3:A34, F42,G3:G34)</f>
+        <v>9.5</v>
+      </c>
+      <c r="H42">
+        <v>10</v>
+      </c>
+      <c r="I42">
+        <f>H42-G42-G43</f>
         <v>0.5</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G32">
-    <sortCondition ref="D3:D32"/>
-    <sortCondition ref="F3:F32"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G33">
+    <sortCondition ref="D3:D33"/>
+    <sortCondition ref="F3:F33"/>
   </sortState>
   <mergeCells count="8">
     <mergeCell ref="H1:K1"/>

</xml_diff>

<commit_message>
Updated Class Diagram and Sprint Backlog
I created new pictures of the class diagrams and updated the sprint
backlog.
</commit_message>
<xml_diff>
--- a/sprints/sprint3/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint3/Sprint Backlog & Burnup Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9e6f5ad0d3e00a8/Desktop/Group5SE2/Group5NutritionTracker/sprints/sprint3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\College Docs\Software Engineering II\Project\Group5NutritionTracker\sprints\sprint3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{AF155070-1F4B-4560-8485-B60514D432E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13E973D7-F7F5-470D-9DDD-35B39FED8F81}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A92A358-D101-4E61-9267-E348E268418C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40635" yWindow="4395" windowWidth="30405" windowHeight="16485" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="39">
   <si>
     <t>Related User Story</t>
   </si>
@@ -74,12 +74,6 @@
     <t>Search Process Client Side</t>
   </si>
   <si>
-    <t>Update DayOfFood Process Client Side</t>
-  </si>
-  <si>
-    <t>Update DayOfFood Process Server Side</t>
-  </si>
-  <si>
     <t>Hookup Add Buttons to Search Page</t>
   </si>
   <si>
@@ -150,6 +144,15 @@
   </si>
   <si>
     <t>Update FoodLog Process Client Side</t>
+  </si>
+  <si>
+    <t>Update FoodLog Process Server Side</t>
+  </si>
+  <si>
+    <t>Change Date of Food Log Client Side</t>
+  </si>
+  <si>
+    <t>Change Date of Food Log Server Side</t>
   </si>
 </sst>
 </file>
@@ -422,16 +425,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>6</c:v>
+                  <c:v>9.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15</c:v>
+                  <c:v>24.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15</c:v>
+                  <c:v>24.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15</c:v>
+                  <c:v>24.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -465,16 +468,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>39.5</c:v>
+                  <c:v>40.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39.5</c:v>
+                  <c:v>40.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>39.5</c:v>
+                  <c:v>40.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>39.5</c:v>
+                  <c:v>40.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1517,31 +1520,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K42"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.54296875" customWidth="1"/>
-    <col min="3" max="3" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" customWidth="1"/>
-    <col min="5" max="5" width="51.453125" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="51.42578125" customWidth="1"/>
     <col min="6" max="6" width="44" customWidth="1"/>
-    <col min="7" max="7" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.81640625" customWidth="1"/>
-    <col min="10" max="10" width="10.7265625" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>9</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>0</v>
@@ -1559,7 +1562,7 @@
       <c r="J1" s="10"/>
       <c r="K1" s="10"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="12"/>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -1580,13 +1583,13 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D3" s="9">
         <v>1.1000000000000001</v>
@@ -1595,7 +1598,7 @@
         <v>10</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G3" s="6">
         <v>3</v>
@@ -1609,12 +1612,14 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B4" s="9"/>
-      <c r="C4" s="6"/>
+      <c r="C4" s="6" t="s">
+        <v>14</v>
+      </c>
       <c r="D4" s="9">
         <v>1.1000000000000001</v>
       </c>
@@ -1627,18 +1632,22 @@
       <c r="G4" s="6">
         <v>2.5</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
+      <c r="H4" s="3">
+        <v>2</v>
+      </c>
+      <c r="I4" s="3">
+        <v>0</v>
+      </c>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D5" s="9">
         <v>1.2</v>
@@ -1647,10 +1656,10 @@
         <v>10</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G5" s="6">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H5" s="3">
         <v>3</v>
@@ -1661,35 +1670,43 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B6" s="9"/>
-      <c r="C6" s="6"/>
+      <c r="C6" s="6" t="s">
+        <v>14</v>
+      </c>
       <c r="D6" s="9">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="G6" s="6">
         <v>2.5</v>
       </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
+      <c r="H6" s="3">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3">
+        <v>1.5</v>
+      </c>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B7" s="9"/>
-      <c r="C7" s="6"/>
+      <c r="C7" s="6" t="s">
+        <v>13</v>
+      </c>
       <c r="D7" s="9">
         <v>1.3</v>
       </c>
@@ -1697,17 +1714,21 @@
         <v>10</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="G7" s="6">
-        <v>2.5</v>
-      </c>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3">
+        <v>2</v>
+      </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>15</v>
       </c>
@@ -1722,212 +1743,238 @@
         <v>10</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G8" s="6">
-        <v>3</v>
-      </c>
-      <c r="H8" s="3">
-        <v>0</v>
-      </c>
-      <c r="I8" s="3">
         <v>2</v>
       </c>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="6"/>
+      <c r="B9" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>14</v>
+      </c>
       <c r="D9" s="9">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="G9" s="6">
-        <v>3</v>
-      </c>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
+        <v>1.5</v>
+      </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B10" s="9"/>
-      <c r="C10" s="6"/>
+      <c r="C10" s="6" t="s">
+        <v>14</v>
+      </c>
       <c r="D10" s="9">
         <v>2.1</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G10" s="6">
-        <v>2</v>
-      </c>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="H10" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="I10" s="3">
+        <v>0</v>
+      </c>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B11" s="9"/>
-      <c r="C11" s="6"/>
+      <c r="C11" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="D11" s="9">
-        <v>2.2000000000000002</v>
+        <v>2.1</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G11" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="9">
-        <v>3.1</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G12" s="6">
-        <v>5</v>
-      </c>
-      <c r="H12" s="3">
-        <v>0</v>
-      </c>
-      <c r="I12" s="3">
         <v>3</v>
       </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="6"/>
+      <c r="B13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>13</v>
+      </c>
       <c r="D13" s="9">
         <v>3.1</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>27</v>
       </c>
       <c r="G13" s="6">
-        <v>2.5</v>
-      </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+        <v>5</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>3</v>
+      </c>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B14" s="9"/>
-      <c r="C14" s="6"/>
+      <c r="C14" s="6" t="s">
+        <v>14</v>
+      </c>
       <c r="D14" s="9">
         <v>3.1</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G14" s="6">
         <v>2.5</v>
       </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
+      <c r="H14" s="3">
+        <v>0</v>
+      </c>
+      <c r="I14" s="3">
+        <v>1.5</v>
+      </c>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="9"/>
+        <v>15</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="C15" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D15" s="9">
         <v>3.1</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G15" s="6">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H15" s="3">
         <v>0</v>
       </c>
       <c r="I15" s="3">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="9"/>
+        <v>16</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="C16" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D16" s="9">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G16" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H16" s="3">
         <v>0</v>
@@ -1938,20 +1985,38 @@
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A17" s="6"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="9">
+        <v>3.2</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" s="6">
+        <v>3</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0</v>
+      </c>
+      <c r="I17" s="3">
+        <v>2</v>
+      </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
       <c r="B18" s="9"/>
       <c r="C18" s="6"/>
@@ -1964,7 +2029,7 @@
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
       <c r="B19" s="9"/>
       <c r="C19" s="6"/>
@@ -1977,7 +2042,7 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
       <c r="B20" s="9"/>
       <c r="C20" s="6"/>
@@ -1990,7 +2055,7 @@
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="6"/>
       <c r="B21" s="9"/>
       <c r="C21" s="6"/>
@@ -2003,7 +2068,7 @@
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="6"/>
       <c r="B22" s="9"/>
       <c r="C22" s="6"/>
@@ -2016,7 +2081,7 @@
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="6"/>
       <c r="B23" s="9"/>
       <c r="C23" s="6"/>
@@ -2029,7 +2094,7 @@
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="6"/>
       <c r="B24" s="9"/>
       <c r="C24" s="6"/>
@@ -2042,7 +2107,7 @@
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="6"/>
       <c r="B25" s="9"/>
       <c r="C25" s="6"/>
@@ -2055,7 +2120,7 @@
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="9"/>
       <c r="C26" s="6"/>
@@ -2068,7 +2133,7 @@
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="9"/>
       <c r="C27" s="6"/>
@@ -2081,7 +2146,7 @@
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
       <c r="B28" s="9"/>
       <c r="C28" s="6"/>
@@ -2094,7 +2159,7 @@
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="6"/>
       <c r="B29" s="9"/>
       <c r="C29" s="6"/>
@@ -2107,7 +2172,7 @@
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
       <c r="B30" s="9"/>
       <c r="C30" s="6"/>
@@ -2120,7 +2185,7 @@
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
       <c r="B31" s="9"/>
       <c r="C31" s="6"/>
@@ -2133,7 +2198,7 @@
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
       <c r="B32" s="9"/>
       <c r="C32" s="6"/>
@@ -2146,7 +2211,7 @@
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="6"/>
       <c r="B33" s="9"/>
       <c r="C33" s="6"/>
@@ -2159,7 +2224,7 @@
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
       <c r="B34" s="9"/>
       <c r="C34" s="6"/>
@@ -2172,7 +2237,7 @@
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -2183,123 +2248,123 @@
       </c>
       <c r="G35" s="5">
         <f>SUM(G3:G34)</f>
-        <v>39.5</v>
+        <v>40.5</v>
       </c>
       <c r="H35" s="5">
         <f>SUM(H3:H34)</f>
-        <v>6</v>
+        <v>9.5</v>
       </c>
       <c r="I35" s="5">
         <f>SUM(I3:I34, H35)</f>
-        <v>15</v>
+        <v>24.5</v>
       </c>
       <c r="J35" s="5">
         <f>SUM(J3:J34, I35)</f>
-        <v>15</v>
+        <v>24.5</v>
       </c>
       <c r="K35" s="5">
         <f>SUM(K3:K34, J35)</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="G36">
         <v>96</v>
       </c>
       <c r="H36">
         <f>$G$35</f>
-        <v>39.5</v>
+        <v>40.5</v>
       </c>
       <c r="I36">
         <f t="shared" ref="I36:K36" si="0">$G$35</f>
-        <v>39.5</v>
+        <v>40.5</v>
       </c>
       <c r="J36">
         <f t="shared" si="0"/>
-        <v>39.5</v>
+        <v>40.5</v>
       </c>
       <c r="K36">
         <f t="shared" si="0"/>
-        <v>39.5</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" ht="58" x14ac:dyDescent="0.35">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="F38" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H38" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="G38" s="7" t="s">
+      <c r="I38" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H38" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="J38" s="8"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F39" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G39">
         <f>SUMIF(A3:A34, F39,G3:G34)</f>
-        <v>8</v>
+        <v>10.5</v>
       </c>
       <c r="H39">
         <v>10</v>
       </c>
       <c r="I39">
         <f>H39-G39-G43</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F40" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G40">
         <f>SUMIF(A3:A34, F40,G3:G34)</f>
-        <v>10</v>
+        <v>9.5</v>
       </c>
       <c r="H40">
         <v>10</v>
       </c>
       <c r="I40">
         <f>H40-G40-G43</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F41" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G41">
         <f>SUMIF(A3:A34, F41,G3:G34)</f>
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="H41">
         <v>10</v>
       </c>
       <c r="I41">
         <f>H41-G41-G43</f>
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F42" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G42">
         <f>SUMIF(A3:A34, F42,G3:G34)</f>
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="H42">
         <v>10</v>
       </c>
       <c r="I42">
         <f>H42-G42-G43</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>